<commit_message>
AYTO VIP 2024 Nacht2
</commit_message>
<xml_diff>
--- a/AYTO_Berechnung/AYTO_Data.xlsx
+++ b/AYTO_Berechnung/AYTO_Data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
   <si>
     <t>ID</t>
   </si>
@@ -217,6 +217,9 @@
   </si>
   <si>
     <t>Matchbox Folge 2/3</t>
+  </si>
+  <si>
+    <t>Matchbox Folge 4/5</t>
   </si>
 </sst>
 </file>
@@ -597,6 +600,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -611,9 +617,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1316,13 +1319,23 @@
       <c r="B5" s="9">
         <v>2</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
+      <c r="C5" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="F5" s="30"/>
-      <c r="G5" s="10"/>
+      <c r="G5" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="H5" s="30"/>
-      <c r="I5" s="7"/>
+      <c r="I5" s="7" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="6" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B6" s="9">
@@ -1714,23 +1727,23 @@
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:16" s="22" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+      <c r="M2" s="46"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="47"/>
     </row>
     <row r="3" spans="1:16" s="23" customFormat="1" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="24"/>
@@ -1770,7 +1783,7 @@
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="25"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="42">
+      <c r="C5" s="43">
         <v>1</v>
       </c>
       <c r="D5" s="12" t="str">
@@ -1822,7 +1835,7 @@
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="25"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="43"/>
+      <c r="C6" s="44"/>
       <c r="D6" s="7" t="s">
         <v>41</v>
       </c>
@@ -1915,7 +1928,7 @@
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="25"/>
       <c r="B10" s="16"/>
-      <c r="C10" s="42">
+      <c r="C10" s="43">
         <v>2</v>
       </c>
       <c r="D10" s="12" t="str">
@@ -1967,19 +1980,41 @@
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="25"/>
       <c r="B11" s="16"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="N11" s="13"/>
-      <c r="O11" s="27"/>
+      <c r="O11" s="27">
+        <v>3</v>
+      </c>
       <c r="P11" s="21"/>
     </row>
     <row r="12" spans="1:16" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2038,7 +2073,7 @@
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="25"/>
       <c r="B15" s="16"/>
-      <c r="C15" s="42">
+      <c r="C15" s="43">
         <v>3</v>
       </c>
       <c r="D15" s="12" t="str">
@@ -2090,7 +2125,7 @@
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="25"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="43"/>
+      <c r="C16" s="44"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
@@ -2161,7 +2196,7 @@
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="42">
+      <c r="C20" s="43">
         <v>4</v>
       </c>
       <c r="D20" s="12" t="str">
@@ -2213,7 +2248,7 @@
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="25"/>
       <c r="B21" s="16"/>
-      <c r="C21" s="43"/>
+      <c r="C21" s="44"/>
       <c r="D21" s="28"/>
       <c r="E21" s="28"/>
       <c r="F21" s="28"/>
@@ -2284,7 +2319,7 @@
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="25"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="42">
+      <c r="C25" s="43">
         <v>5</v>
       </c>
       <c r="D25" s="12" t="str">
@@ -2336,7 +2371,7 @@
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="25"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="43"/>
+      <c r="C26" s="44"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
@@ -2407,7 +2442,7 @@
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="25"/>
       <c r="B30" s="16"/>
-      <c r="C30" s="42">
+      <c r="C30" s="43">
         <v>6</v>
       </c>
       <c r="D30" s="12" t="str">
@@ -2459,7 +2494,7 @@
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="25"/>
       <c r="B31" s="16"/>
-      <c r="C31" s="43"/>
+      <c r="C31" s="44"/>
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
@@ -2530,7 +2565,7 @@
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
       <c r="B35" s="16"/>
-      <c r="C35" s="42">
+      <c r="C35" s="43">
         <v>7</v>
       </c>
       <c r="D35" s="12" t="str">
@@ -2582,7 +2617,7 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="25"/>
       <c r="B36" s="16"/>
-      <c r="C36" s="43"/>
+      <c r="C36" s="44"/>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
@@ -2653,7 +2688,7 @@
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="25"/>
       <c r="B40" s="16"/>
-      <c r="C40" s="42">
+      <c r="C40" s="43">
         <v>8</v>
       </c>
       <c r="D40" s="12" t="str">
@@ -2705,7 +2740,7 @@
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="25"/>
       <c r="B41" s="16"/>
-      <c r="C41" s="43"/>
+      <c r="C41" s="44"/>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
@@ -2776,7 +2811,7 @@
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="25"/>
       <c r="B45" s="16"/>
-      <c r="C45" s="42">
+      <c r="C45" s="43">
         <v>9</v>
       </c>
       <c r="D45" s="12" t="str">
@@ -2828,7 +2863,7 @@
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="25"/>
       <c r="B46" s="16"/>
-      <c r="C46" s="43"/>
+      <c r="C46" s="44"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
@@ -2899,7 +2934,7 @@
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="25"/>
       <c r="B50" s="16"/>
-      <c r="C50" s="42">
+      <c r="C50" s="43">
         <v>10</v>
       </c>
       <c r="D50" s="12" t="str">
@@ -2951,7 +2986,7 @@
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="25"/>
       <c r="B51" s="16"/>
-      <c r="C51" s="43"/>
+      <c r="C51" s="44"/>
       <c r="D51" s="7"/>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
@@ -2986,42 +3021,42 @@
     </row>
     <row r="53" spans="1:16" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B54" s="47" t="s">
+      <c r="B54" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C54" s="47"/>
-      <c r="D54" s="47"/>
-      <c r="E54" s="47"/>
-      <c r="F54" s="47"/>
-      <c r="G54" s="47"/>
-      <c r="H54" s="47"/>
-      <c r="I54" s="47"/>
-      <c r="J54" s="47"/>
-      <c r="K54" s="47"/>
-      <c r="L54" s="47"/>
-      <c r="M54" s="47"/>
-      <c r="N54" s="47"/>
-      <c r="O54" s="47"/>
-      <c r="P54" s="47"/>
+      <c r="C54" s="42"/>
+      <c r="D54" s="42"/>
+      <c r="E54" s="42"/>
+      <c r="F54" s="42"/>
+      <c r="G54" s="42"/>
+      <c r="H54" s="42"/>
+      <c r="I54" s="42"/>
+      <c r="J54" s="42"/>
+      <c r="K54" s="42"/>
+      <c r="L54" s="42"/>
+      <c r="M54" s="42"/>
+      <c r="N54" s="42"/>
+      <c r="O54" s="42"/>
+      <c r="P54" s="42"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B55" s="47" t="s">
+      <c r="B55" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C55" s="47"/>
-      <c r="D55" s="47"/>
-      <c r="E55" s="47"/>
-      <c r="F55" s="47"/>
-      <c r="G55" s="47"/>
-      <c r="H55" s="47"/>
-      <c r="I55" s="47"/>
-      <c r="J55" s="47"/>
-      <c r="K55" s="47"/>
-      <c r="L55" s="47"/>
-      <c r="M55" s="47"/>
-      <c r="N55" s="47"/>
-      <c r="O55" s="47"/>
-      <c r="P55" s="47"/>
+      <c r="C55" s="42"/>
+      <c r="D55" s="42"/>
+      <c r="E55" s="42"/>
+      <c r="F55" s="42"/>
+      <c r="G55" s="42"/>
+      <c r="H55" s="42"/>
+      <c r="I55" s="42"/>
+      <c r="J55" s="42"/>
+      <c r="K55" s="42"/>
+      <c r="L55" s="42"/>
+      <c r="M55" s="42"/>
+      <c r="N55" s="42"/>
+      <c r="O55" s="42"/>
+      <c r="P55" s="42"/>
     </row>
   </sheetData>
   <sheetProtection password="CA39" sheet="1" objects="1" scenarios="1"/>
@@ -3029,12 +3064,6 @@
     <protectedRange sqref="D6:O6 D11:O11 D16:O16 D21:O21 D26:O26 D31:O31 D36:O36 D41:O41 D46:O46 D51:O51" name="Bereich1"/>
   </protectedRanges>
   <mergeCells count="13">
-    <mergeCell ref="B54:P54"/>
-    <mergeCell ref="B55:P55"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="C35:C36"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="C25:C26"/>
@@ -3042,6 +3071,12 @@
     <mergeCell ref="C40:C41"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B54:P54"/>
+    <mergeCell ref="B55:P55"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="C35:C36"/>
   </mergeCells>
   <conditionalFormatting sqref="D16:M16 D11:M11 D6:M6 D26:M26 D31:M31 D36:M36 D41:M41 D46:M46 D51:M51 D21:M21">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="notEqual">

</xml_diff>

<commit_message>
AYTO VIP 2024 Nacht 3
</commit_message>
<xml_diff>
--- a/AYTO_Berechnung/AYTO_Data.xlsx
+++ b/AYTO_Berechnung/AYTO_Data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="53">
   <si>
     <t>ID</t>
   </si>
@@ -219,7 +219,7 @@
     <t>Matchbox Folge 2/3</t>
   </si>
   <si>
-    <t>Matchbox Folge 4/5</t>
+    <t>Matchbox Folge 4/5 (Folge 6/7 verkauft)</t>
   </si>
 </sst>
 </file>
@@ -2126,18 +2126,40 @@
       <c r="A16" s="25"/>
       <c r="B16" s="16"/>
       <c r="C16" s="44"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
+      <c r="D16" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>35</v>
+      </c>
       <c r="N16" s="13"/>
-      <c r="O16" s="27"/>
+      <c r="O16" s="27">
+        <v>3</v>
+      </c>
       <c r="P16" s="21"/>
     </row>
     <row r="17" spans="1:16" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
AYTO VIP 2024 Nacht 4
</commit_message>
<xml_diff>
--- a/AYTO_Berechnung/AYTO_Data.xlsx
+++ b/AYTO_Berechnung/AYTO_Data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="54">
   <si>
     <t>ID</t>
   </si>
@@ -220,6 +220,9 @@
   </si>
   <si>
     <t>Matchbox Folge 4/5 (Folge 6/7 verkauft)</t>
+  </si>
+  <si>
+    <t>Matchbox Folge 8/9</t>
   </si>
 </sst>
 </file>
@@ -1341,13 +1344,21 @@
       <c r="B6" s="9">
         <v>3</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
+      <c r="C6" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>12</v>
+      </c>
       <c r="F6" s="30"/>
       <c r="G6" s="10"/>
       <c r="H6" s="30"/>
-      <c r="I6" s="7"/>
+      <c r="I6" s="7" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="7" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B7" s="9">
@@ -2271,18 +2282,40 @@
       <c r="A21" s="25"/>
       <c r="B21" s="16"/>
       <c r="C21" s="44"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
-      <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
+      <c r="D21" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="G21" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="H21" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="I21" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="J21" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="K21" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="L21" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="M21" s="28" t="s">
+        <v>41</v>
+      </c>
       <c r="N21" s="13"/>
-      <c r="O21" s="27"/>
+      <c r="O21" s="27">
+        <v>1</v>
+      </c>
       <c r="P21" s="21"/>
     </row>
     <row r="22" spans="1:16" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
AYTO VIP 2024 Nacht 5
</commit_message>
<xml_diff>
--- a/AYTO_Berechnung/AYTO_Data.xlsx
+++ b/AYTO_Berechnung/AYTO_Data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="54">
   <si>
     <t>ID</t>
   </si>
@@ -222,7 +222,7 @@
     <t>Matchbox Folge 4/5 (Folge 6/7 verkauft)</t>
   </si>
   <si>
-    <t>Matchbox Folge 8/9</t>
+    <t>Matchbox Folge 8/9 (Folge 10/11 verkauft)</t>
   </si>
 </sst>
 </file>
@@ -603,23 +603,23 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1738,23 +1738,23 @@
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:16" s="22" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="47"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="46"/>
     </row>
     <row r="3" spans="1:16" s="23" customFormat="1" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="24"/>
@@ -1794,7 +1794,7 @@
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="25"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="43">
+      <c r="C5" s="42">
         <v>1</v>
       </c>
       <c r="D5" s="12" t="str">
@@ -1846,7 +1846,7 @@
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="25"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="44"/>
+      <c r="C6" s="43"/>
       <c r="D6" s="7" t="s">
         <v>41</v>
       </c>
@@ -1939,7 +1939,7 @@
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="25"/>
       <c r="B10" s="16"/>
-      <c r="C10" s="43">
+      <c r="C10" s="42">
         <v>2</v>
       </c>
       <c r="D10" s="12" t="str">
@@ -1991,7 +1991,7 @@
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="25"/>
       <c r="B11" s="16"/>
-      <c r="C11" s="44"/>
+      <c r="C11" s="43"/>
       <c r="D11" s="7" t="s">
         <v>38</v>
       </c>
@@ -2084,7 +2084,7 @@
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="25"/>
       <c r="B15" s="16"/>
-      <c r="C15" s="43">
+      <c r="C15" s="42">
         <v>3</v>
       </c>
       <c r="D15" s="12" t="str">
@@ -2136,7 +2136,7 @@
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="25"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="44"/>
+      <c r="C16" s="43"/>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
@@ -2229,7 +2229,7 @@
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="43">
+      <c r="C20" s="42">
         <v>4</v>
       </c>
       <c r="D20" s="12" t="str">
@@ -2281,7 +2281,7 @@
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="25"/>
       <c r="B21" s="16"/>
-      <c r="C21" s="44"/>
+      <c r="C21" s="43"/>
       <c r="D21" s="28" t="s">
         <v>38</v>
       </c>
@@ -2374,7 +2374,7 @@
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="25"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="43">
+      <c r="C25" s="42">
         <v>5</v>
       </c>
       <c r="D25" s="12" t="str">
@@ -2426,19 +2426,41 @@
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="25"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
+      <c r="C26" s="43"/>
+      <c r="D26" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="N26" s="13"/>
-      <c r="O26" s="27"/>
+      <c r="O26" s="27">
+        <v>5</v>
+      </c>
       <c r="P26" s="21"/>
     </row>
     <row r="27" spans="1:16" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2497,7 +2519,7 @@
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="25"/>
       <c r="B30" s="16"/>
-      <c r="C30" s="43">
+      <c r="C30" s="42">
         <v>6</v>
       </c>
       <c r="D30" s="12" t="str">
@@ -2549,7 +2571,7 @@
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="25"/>
       <c r="B31" s="16"/>
-      <c r="C31" s="44"/>
+      <c r="C31" s="43"/>
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
@@ -2620,7 +2642,7 @@
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
       <c r="B35" s="16"/>
-      <c r="C35" s="43">
+      <c r="C35" s="42">
         <v>7</v>
       </c>
       <c r="D35" s="12" t="str">
@@ -2672,7 +2694,7 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="25"/>
       <c r="B36" s="16"/>
-      <c r="C36" s="44"/>
+      <c r="C36" s="43"/>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
@@ -2743,7 +2765,7 @@
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="25"/>
       <c r="B40" s="16"/>
-      <c r="C40" s="43">
+      <c r="C40" s="42">
         <v>8</v>
       </c>
       <c r="D40" s="12" t="str">
@@ -2795,7 +2817,7 @@
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="25"/>
       <c r="B41" s="16"/>
-      <c r="C41" s="44"/>
+      <c r="C41" s="43"/>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
@@ -2866,7 +2888,7 @@
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="25"/>
       <c r="B45" s="16"/>
-      <c r="C45" s="43">
+      <c r="C45" s="42">
         <v>9</v>
       </c>
       <c r="D45" s="12" t="str">
@@ -2918,7 +2940,7 @@
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="25"/>
       <c r="B46" s="16"/>
-      <c r="C46" s="44"/>
+      <c r="C46" s="43"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
@@ -2989,7 +3011,7 @@
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="25"/>
       <c r="B50" s="16"/>
-      <c r="C50" s="43">
+      <c r="C50" s="42">
         <v>10</v>
       </c>
       <c r="D50" s="12" t="str">
@@ -3041,7 +3063,7 @@
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="25"/>
       <c r="B51" s="16"/>
-      <c r="C51" s="44"/>
+      <c r="C51" s="43"/>
       <c r="D51" s="7"/>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
@@ -3076,42 +3098,42 @@
     </row>
     <row r="53" spans="1:16" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B54" s="42" t="s">
+      <c r="B54" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C54" s="42"/>
-      <c r="D54" s="42"/>
-      <c r="E54" s="42"/>
-      <c r="F54" s="42"/>
-      <c r="G54" s="42"/>
-      <c r="H54" s="42"/>
-      <c r="I54" s="42"/>
-      <c r="J54" s="42"/>
-      <c r="K54" s="42"/>
-      <c r="L54" s="42"/>
-      <c r="M54" s="42"/>
-      <c r="N54" s="42"/>
-      <c r="O54" s="42"/>
-      <c r="P54" s="42"/>
+      <c r="C54" s="47"/>
+      <c r="D54" s="47"/>
+      <c r="E54" s="47"/>
+      <c r="F54" s="47"/>
+      <c r="G54" s="47"/>
+      <c r="H54" s="47"/>
+      <c r="I54" s="47"/>
+      <c r="J54" s="47"/>
+      <c r="K54" s="47"/>
+      <c r="L54" s="47"/>
+      <c r="M54" s="47"/>
+      <c r="N54" s="47"/>
+      <c r="O54" s="47"/>
+      <c r="P54" s="47"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B55" s="42" t="s">
+      <c r="B55" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C55" s="42"/>
-      <c r="D55" s="42"/>
-      <c r="E55" s="42"/>
-      <c r="F55" s="42"/>
-      <c r="G55" s="42"/>
-      <c r="H55" s="42"/>
-      <c r="I55" s="42"/>
-      <c r="J55" s="42"/>
-      <c r="K55" s="42"/>
-      <c r="L55" s="42"/>
-      <c r="M55" s="42"/>
-      <c r="N55" s="42"/>
-      <c r="O55" s="42"/>
-      <c r="P55" s="42"/>
+      <c r="C55" s="47"/>
+      <c r="D55" s="47"/>
+      <c r="E55" s="47"/>
+      <c r="F55" s="47"/>
+      <c r="G55" s="47"/>
+      <c r="H55" s="47"/>
+      <c r="I55" s="47"/>
+      <c r="J55" s="47"/>
+      <c r="K55" s="47"/>
+      <c r="L55" s="47"/>
+      <c r="M55" s="47"/>
+      <c r="N55" s="47"/>
+      <c r="O55" s="47"/>
+      <c r="P55" s="47"/>
     </row>
   </sheetData>
   <sheetProtection password="CA39" sheet="1" objects="1" scenarios="1"/>
@@ -3119,6 +3141,12 @@
     <protectedRange sqref="D6:O6 D11:O11 D16:O16 D21:O21 D26:O26 D31:O31 D36:O36 D41:O41 D46:O46 D51:O51" name="Bereich1"/>
   </protectedRanges>
   <mergeCells count="13">
+    <mergeCell ref="B54:P54"/>
+    <mergeCell ref="B55:P55"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="C35:C36"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="C25:C26"/>
@@ -3126,12 +3154,6 @@
     <mergeCell ref="C40:C41"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B54:P54"/>
-    <mergeCell ref="B55:P55"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="C35:C36"/>
   </mergeCells>
   <conditionalFormatting sqref="D16:M16 D11:M11 D6:M6 D26:M26 D31:M31 D36:M36 D41:M41 D46:M46 D51:M51 D21:M21">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="notEqual">

</xml_diff>

<commit_message>
AYTO VIP 2024 Nacht 6
</commit_message>
<xml_diff>
--- a/AYTO_Berechnung/AYTO_Data.xlsx
+++ b/AYTO_Berechnung/AYTO_Data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="55">
   <si>
     <t>ID</t>
   </si>
@@ -223,6 +223,9 @@
   </si>
   <si>
     <t>Matchbox Folge 8/9 (Folge 10/11 verkauft)</t>
+  </si>
+  <si>
+    <t>Matchbox Folge 12/13</t>
   </si>
 </sst>
 </file>
@@ -603,6 +606,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -617,9 +623,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1364,13 +1367,23 @@
       <c r="B7" s="9">
         <v>4</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
+      <c r="C7" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="F7" s="30"/>
-      <c r="G7" s="10"/>
+      <c r="G7" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="H7" s="30"/>
-      <c r="I7" s="7"/>
+      <c r="I7" s="7" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="8" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B8" s="9">
@@ -1738,23 +1751,23 @@
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:16" s="22" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+      <c r="M2" s="46"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="47"/>
     </row>
     <row r="3" spans="1:16" s="23" customFormat="1" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="24"/>
@@ -1794,7 +1807,7 @@
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="25"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="42">
+      <c r="C5" s="43">
         <v>1</v>
       </c>
       <c r="D5" s="12" t="str">
@@ -1846,7 +1859,7 @@
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="25"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="43"/>
+      <c r="C6" s="44"/>
       <c r="D6" s="7" t="s">
         <v>41</v>
       </c>
@@ -1939,7 +1952,7 @@
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="25"/>
       <c r="B10" s="16"/>
-      <c r="C10" s="42">
+      <c r="C10" s="43">
         <v>2</v>
       </c>
       <c r="D10" s="12" t="str">
@@ -1991,7 +2004,7 @@
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="25"/>
       <c r="B11" s="16"/>
-      <c r="C11" s="43"/>
+      <c r="C11" s="44"/>
       <c r="D11" s="7" t="s">
         <v>38</v>
       </c>
@@ -2084,7 +2097,7 @@
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="25"/>
       <c r="B15" s="16"/>
-      <c r="C15" s="42">
+      <c r="C15" s="43">
         <v>3</v>
       </c>
       <c r="D15" s="12" t="str">
@@ -2136,7 +2149,7 @@
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="25"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="43"/>
+      <c r="C16" s="44"/>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
@@ -2229,7 +2242,7 @@
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="42">
+      <c r="C20" s="43">
         <v>4</v>
       </c>
       <c r="D20" s="12" t="str">
@@ -2281,7 +2294,7 @@
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="25"/>
       <c r="B21" s="16"/>
-      <c r="C21" s="43"/>
+      <c r="C21" s="44"/>
       <c r="D21" s="28" t="s">
         <v>38</v>
       </c>
@@ -2374,7 +2387,7 @@
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="25"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="42">
+      <c r="C25" s="43">
         <v>5</v>
       </c>
       <c r="D25" s="12" t="str">
@@ -2426,7 +2439,7 @@
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="25"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="43"/>
+      <c r="C26" s="44"/>
       <c r="D26" s="7" t="s">
         <v>37</v>
       </c>
@@ -2519,7 +2532,7 @@
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="25"/>
       <c r="B30" s="16"/>
-      <c r="C30" s="42">
+      <c r="C30" s="43">
         <v>6</v>
       </c>
       <c r="D30" s="12" t="str">
@@ -2571,19 +2584,41 @@
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="25"/>
       <c r="B31" s="16"/>
-      <c r="C31" s="43"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="M31" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="N31" s="13"/>
-      <c r="O31" s="27"/>
+      <c r="O31" s="27">
+        <v>6</v>
+      </c>
       <c r="P31" s="21"/>
     </row>
     <row r="32" spans="1:16" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2642,7 +2677,7 @@
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
       <c r="B35" s="16"/>
-      <c r="C35" s="42">
+      <c r="C35" s="43">
         <v>7</v>
       </c>
       <c r="D35" s="12" t="str">
@@ -2694,7 +2729,7 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="25"/>
       <c r="B36" s="16"/>
-      <c r="C36" s="43"/>
+      <c r="C36" s="44"/>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
@@ -2765,7 +2800,7 @@
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="25"/>
       <c r="B40" s="16"/>
-      <c r="C40" s="42">
+      <c r="C40" s="43">
         <v>8</v>
       </c>
       <c r="D40" s="12" t="str">
@@ -2817,7 +2852,7 @@
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="25"/>
       <c r="B41" s="16"/>
-      <c r="C41" s="43"/>
+      <c r="C41" s="44"/>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
@@ -2888,7 +2923,7 @@
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="25"/>
       <c r="B45" s="16"/>
-      <c r="C45" s="42">
+      <c r="C45" s="43">
         <v>9</v>
       </c>
       <c r="D45" s="12" t="str">
@@ -2940,7 +2975,7 @@
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="25"/>
       <c r="B46" s="16"/>
-      <c r="C46" s="43"/>
+      <c r="C46" s="44"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
@@ -3011,7 +3046,7 @@
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="25"/>
       <c r="B50" s="16"/>
-      <c r="C50" s="42">
+      <c r="C50" s="43">
         <v>10</v>
       </c>
       <c r="D50" s="12" t="str">
@@ -3063,7 +3098,7 @@
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="25"/>
       <c r="B51" s="16"/>
-      <c r="C51" s="43"/>
+      <c r="C51" s="44"/>
       <c r="D51" s="7"/>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
@@ -3098,42 +3133,42 @@
     </row>
     <row r="53" spans="1:16" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B54" s="47" t="s">
+      <c r="B54" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C54" s="47"/>
-      <c r="D54" s="47"/>
-      <c r="E54" s="47"/>
-      <c r="F54" s="47"/>
-      <c r="G54" s="47"/>
-      <c r="H54" s="47"/>
-      <c r="I54" s="47"/>
-      <c r="J54" s="47"/>
-      <c r="K54" s="47"/>
-      <c r="L54" s="47"/>
-      <c r="M54" s="47"/>
-      <c r="N54" s="47"/>
-      <c r="O54" s="47"/>
-      <c r="P54" s="47"/>
+      <c r="C54" s="42"/>
+      <c r="D54" s="42"/>
+      <c r="E54" s="42"/>
+      <c r="F54" s="42"/>
+      <c r="G54" s="42"/>
+      <c r="H54" s="42"/>
+      <c r="I54" s="42"/>
+      <c r="J54" s="42"/>
+      <c r="K54" s="42"/>
+      <c r="L54" s="42"/>
+      <c r="M54" s="42"/>
+      <c r="N54" s="42"/>
+      <c r="O54" s="42"/>
+      <c r="P54" s="42"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B55" s="47" t="s">
+      <c r="B55" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C55" s="47"/>
-      <c r="D55" s="47"/>
-      <c r="E55" s="47"/>
-      <c r="F55" s="47"/>
-      <c r="G55" s="47"/>
-      <c r="H55" s="47"/>
-      <c r="I55" s="47"/>
-      <c r="J55" s="47"/>
-      <c r="K55" s="47"/>
-      <c r="L55" s="47"/>
-      <c r="M55" s="47"/>
-      <c r="N55" s="47"/>
-      <c r="O55" s="47"/>
-      <c r="P55" s="47"/>
+      <c r="C55" s="42"/>
+      <c r="D55" s="42"/>
+      <c r="E55" s="42"/>
+      <c r="F55" s="42"/>
+      <c r="G55" s="42"/>
+      <c r="H55" s="42"/>
+      <c r="I55" s="42"/>
+      <c r="J55" s="42"/>
+      <c r="K55" s="42"/>
+      <c r="L55" s="42"/>
+      <c r="M55" s="42"/>
+      <c r="N55" s="42"/>
+      <c r="O55" s="42"/>
+      <c r="P55" s="42"/>
     </row>
   </sheetData>
   <sheetProtection password="CA39" sheet="1" objects="1" scenarios="1"/>
@@ -3141,12 +3176,6 @@
     <protectedRange sqref="D6:O6 D11:O11 D16:O16 D21:O21 D26:O26 D31:O31 D36:O36 D41:O41 D46:O46 D51:O51" name="Bereich1"/>
   </protectedRanges>
   <mergeCells count="13">
-    <mergeCell ref="B54:P54"/>
-    <mergeCell ref="B55:P55"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="C35:C36"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="C25:C26"/>
@@ -3154,6 +3183,12 @@
     <mergeCell ref="C40:C41"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B54:P54"/>
+    <mergeCell ref="B55:P55"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="C35:C36"/>
   </mergeCells>
   <conditionalFormatting sqref="D16:M16 D11:M11 D6:M6 D26:M26 D31:M31 D36:M36 D41:M41 D46:M46 D51:M51 D21:M21">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="notEqual">

</xml_diff>

<commit_message>
AYTO VIP 2024 Nacht 7
</commit_message>
<xml_diff>
--- a/AYTO_Berechnung/AYTO_Data.xlsx
+++ b/AYTO_Berechnung/AYTO_Data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="56">
   <si>
     <t>ID</t>
   </si>
@@ -226,6 +226,9 @@
   </si>
   <si>
     <t>Matchbox Folge 12/13</t>
+  </si>
+  <si>
+    <t>Folge 14/15</t>
   </si>
 </sst>
 </file>
@@ -606,23 +609,23 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1389,13 +1392,21 @@
       <c r="B8" s="9">
         <v>5</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
+      <c r="C8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>12</v>
+      </c>
       <c r="F8" s="30"/>
       <c r="G8" s="10"/>
       <c r="H8" s="30"/>
-      <c r="I8" s="7"/>
+      <c r="I8" s="7" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="9" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B9" s="9">
@@ -1751,23 +1762,23 @@
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:16" s="22" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="47"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="46"/>
     </row>
     <row r="3" spans="1:16" s="23" customFormat="1" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="24"/>
@@ -1807,7 +1818,7 @@
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="25"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="43">
+      <c r="C5" s="42">
         <v>1</v>
       </c>
       <c r="D5" s="12" t="str">
@@ -1859,7 +1870,7 @@
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="25"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="44"/>
+      <c r="C6" s="43"/>
       <c r="D6" s="7" t="s">
         <v>41</v>
       </c>
@@ -1952,7 +1963,7 @@
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="25"/>
       <c r="B10" s="16"/>
-      <c r="C10" s="43">
+      <c r="C10" s="42">
         <v>2</v>
       </c>
       <c r="D10" s="12" t="str">
@@ -2004,7 +2015,7 @@
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="25"/>
       <c r="B11" s="16"/>
-      <c r="C11" s="44"/>
+      <c r="C11" s="43"/>
       <c r="D11" s="7" t="s">
         <v>38</v>
       </c>
@@ -2097,7 +2108,7 @@
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="25"/>
       <c r="B15" s="16"/>
-      <c r="C15" s="43">
+      <c r="C15" s="42">
         <v>3</v>
       </c>
       <c r="D15" s="12" t="str">
@@ -2149,7 +2160,7 @@
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="25"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="44"/>
+      <c r="C16" s="43"/>
       <c r="D16" s="7" t="s">
         <v>31</v>
       </c>
@@ -2242,7 +2253,7 @@
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="43">
+      <c r="C20" s="42">
         <v>4</v>
       </c>
       <c r="D20" s="12" t="str">
@@ -2294,7 +2305,7 @@
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="25"/>
       <c r="B21" s="16"/>
-      <c r="C21" s="44"/>
+      <c r="C21" s="43"/>
       <c r="D21" s="28" t="s">
         <v>38</v>
       </c>
@@ -2387,7 +2398,7 @@
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="25"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="43">
+      <c r="C25" s="42">
         <v>5</v>
       </c>
       <c r="D25" s="12" t="str">
@@ -2439,7 +2450,7 @@
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="25"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="44"/>
+      <c r="C26" s="43"/>
       <c r="D26" s="7" t="s">
         <v>37</v>
       </c>
@@ -2532,7 +2543,7 @@
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="25"/>
       <c r="B30" s="16"/>
-      <c r="C30" s="43">
+      <c r="C30" s="42">
         <v>6</v>
       </c>
       <c r="D30" s="12" t="str">
@@ -2584,7 +2595,7 @@
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="25"/>
       <c r="B31" s="16"/>
-      <c r="C31" s="44"/>
+      <c r="C31" s="43"/>
       <c r="D31" s="7" t="s">
         <v>37</v>
       </c>
@@ -2677,7 +2688,7 @@
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
       <c r="B35" s="16"/>
-      <c r="C35" s="43">
+      <c r="C35" s="42">
         <v>7</v>
       </c>
       <c r="D35" s="12" t="str">
@@ -2729,19 +2740,41 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="25"/>
       <c r="B36" s="16"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
-      <c r="L36" s="7"/>
-      <c r="M36" s="7"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I36" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="J36" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K36" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="L36" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="M36" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="N36" s="13"/>
-      <c r="O36" s="27"/>
+      <c r="O36" s="27">
+        <v>6</v>
+      </c>
       <c r="P36" s="21"/>
     </row>
     <row r="37" spans="1:16" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2800,7 +2833,7 @@
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="25"/>
       <c r="B40" s="16"/>
-      <c r="C40" s="43">
+      <c r="C40" s="42">
         <v>8</v>
       </c>
       <c r="D40" s="12" t="str">
@@ -2852,7 +2885,7 @@
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="25"/>
       <c r="B41" s="16"/>
-      <c r="C41" s="44"/>
+      <c r="C41" s="43"/>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
@@ -2923,7 +2956,7 @@
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="25"/>
       <c r="B45" s="16"/>
-      <c r="C45" s="43">
+      <c r="C45" s="42">
         <v>9</v>
       </c>
       <c r="D45" s="12" t="str">
@@ -2975,7 +3008,7 @@
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="25"/>
       <c r="B46" s="16"/>
-      <c r="C46" s="44"/>
+      <c r="C46" s="43"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
@@ -3046,7 +3079,7 @@
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="25"/>
       <c r="B50" s="16"/>
-      <c r="C50" s="43">
+      <c r="C50" s="42">
         <v>10</v>
       </c>
       <c r="D50" s="12" t="str">
@@ -3098,7 +3131,7 @@
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="25"/>
       <c r="B51" s="16"/>
-      <c r="C51" s="44"/>
+      <c r="C51" s="43"/>
       <c r="D51" s="7"/>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
@@ -3133,42 +3166,42 @@
     </row>
     <row r="53" spans="1:16" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B54" s="42" t="s">
+      <c r="B54" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C54" s="42"/>
-      <c r="D54" s="42"/>
-      <c r="E54" s="42"/>
-      <c r="F54" s="42"/>
-      <c r="G54" s="42"/>
-      <c r="H54" s="42"/>
-      <c r="I54" s="42"/>
-      <c r="J54" s="42"/>
-      <c r="K54" s="42"/>
-      <c r="L54" s="42"/>
-      <c r="M54" s="42"/>
-      <c r="N54" s="42"/>
-      <c r="O54" s="42"/>
-      <c r="P54" s="42"/>
+      <c r="C54" s="47"/>
+      <c r="D54" s="47"/>
+      <c r="E54" s="47"/>
+      <c r="F54" s="47"/>
+      <c r="G54" s="47"/>
+      <c r="H54" s="47"/>
+      <c r="I54" s="47"/>
+      <c r="J54" s="47"/>
+      <c r="K54" s="47"/>
+      <c r="L54" s="47"/>
+      <c r="M54" s="47"/>
+      <c r="N54" s="47"/>
+      <c r="O54" s="47"/>
+      <c r="P54" s="47"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B55" s="42" t="s">
+      <c r="B55" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C55" s="42"/>
-      <c r="D55" s="42"/>
-      <c r="E55" s="42"/>
-      <c r="F55" s="42"/>
-      <c r="G55" s="42"/>
-      <c r="H55" s="42"/>
-      <c r="I55" s="42"/>
-      <c r="J55" s="42"/>
-      <c r="K55" s="42"/>
-      <c r="L55" s="42"/>
-      <c r="M55" s="42"/>
-      <c r="N55" s="42"/>
-      <c r="O55" s="42"/>
-      <c r="P55" s="42"/>
+      <c r="C55" s="47"/>
+      <c r="D55" s="47"/>
+      <c r="E55" s="47"/>
+      <c r="F55" s="47"/>
+      <c r="G55" s="47"/>
+      <c r="H55" s="47"/>
+      <c r="I55" s="47"/>
+      <c r="J55" s="47"/>
+      <c r="K55" s="47"/>
+      <c r="L55" s="47"/>
+      <c r="M55" s="47"/>
+      <c r="N55" s="47"/>
+      <c r="O55" s="47"/>
+      <c r="P55" s="47"/>
     </row>
   </sheetData>
   <sheetProtection password="CA39" sheet="1" objects="1" scenarios="1"/>
@@ -3176,6 +3209,12 @@
     <protectedRange sqref="D6:O6 D11:O11 D16:O16 D21:O21 D26:O26 D31:O31 D36:O36 D41:O41 D46:O46 D51:O51" name="Bereich1"/>
   </protectedRanges>
   <mergeCells count="13">
+    <mergeCell ref="B54:P54"/>
+    <mergeCell ref="B55:P55"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="C35:C36"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="C25:C26"/>
@@ -3183,12 +3222,6 @@
     <mergeCell ref="C40:C41"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B54:P54"/>
-    <mergeCell ref="B55:P55"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="C35:C36"/>
   </mergeCells>
   <conditionalFormatting sqref="D16:M16 D11:M11 D6:M6 D26:M26 D31:M31 D36:M36 D41:M41 D46:M46 D51:M51 D21:M21">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="notEqual">

</xml_diff>